<commit_message>
Added keyboard navigation, command palette, reports UI and toast notifications
</commit_message>
<xml_diff>
--- a/backend/generated_reports/sales_report.xlsx
+++ b/backend/generated_reports/sales_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -502,6 +502,33 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>INV-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>495</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2475</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>28-06-2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>